<commit_message>
Record macOS Office and WPS native acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/verification/microsoft-parity/ui-excel-01/parity-excel-ui.xlsx
+++ b/docs/verification/microsoft-parity/ui-excel-01/parity-excel-ui.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neomei/Library/Containers/com.microsoft.Excel/Data/tmp/wpscomposer/session-ghmqgvaj/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neomei/项目/codexprojects/WpsComposer/.worktrees/office-description/docs/verification/microsoft-parity/ui-excel-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{583E8D45-4220-FE44-A323-2A810BCA437F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D5CFD8-1EF8-D240-BB69-72FC9C9F08D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3880" yWindow="3060" windowWidth="27240" windowHeight="16360" xr2:uid="{6A901168-9DBC-FC4A-8B3F-168D71BA5F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Native created" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -131,14 +131,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -660,34 +660,34 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <f>B4*2</f>
         <v>24</v>
       </c>

</xml_diff>